<commit_message>
attendance on sept 7th
</commit_message>
<xml_diff>
--- a/Meeting_Attendance.xlsx
+++ b/Meeting_Attendance.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,38 +425,43 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F45"/>
+  <dimension ref="A1:G45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Register number</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Phone number</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Username</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Member Type</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Meeting 2026-08-28</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Meeting 2026-09-07</t>
         </is>
       </c>
     </row>
@@ -475,6 +492,9 @@
       <c r="F2" t="n">
         <v>0</v>
       </c>
+      <c r="G2" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -503,6 +523,9 @@
       <c r="F3" t="n">
         <v>0</v>
       </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -531,6 +554,9 @@
       <c r="F4" t="n">
         <v>0</v>
       </c>
+      <c r="G4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -559,6 +585,9 @@
       <c r="F5" t="n">
         <v>0</v>
       </c>
+      <c r="G5" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -587,6 +616,9 @@
       <c r="F6" t="n">
         <v>1</v>
       </c>
+      <c r="G6" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -615,6 +647,9 @@
       <c r="F7" t="n">
         <v>0</v>
       </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -643,6 +678,9 @@
       <c r="F8" t="n">
         <v>0</v>
       </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -671,6 +709,9 @@
       <c r="F9" t="n">
         <v>1</v>
       </c>
+      <c r="G9" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -699,6 +740,9 @@
       <c r="F10" t="n">
         <v>1</v>
       </c>
+      <c r="G10" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -727,6 +771,9 @@
       <c r="F11" t="n">
         <v>0</v>
       </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -755,6 +802,9 @@
       <c r="F12" t="n">
         <v>0</v>
       </c>
+      <c r="G12" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -783,6 +833,9 @@
       <c r="F13" t="n">
         <v>0</v>
       </c>
+      <c r="G13" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -811,6 +864,9 @@
       <c r="F14" t="n">
         <v>1</v>
       </c>
+      <c r="G14" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -839,6 +895,9 @@
       <c r="F15" t="n">
         <v>1</v>
       </c>
+      <c r="G15" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -867,6 +926,9 @@
       <c r="F16" t="n">
         <v>1</v>
       </c>
+      <c r="G16" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -895,6 +957,9 @@
       <c r="F17" t="n">
         <v>0</v>
       </c>
+      <c r="G17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -923,6 +988,9 @@
       <c r="F18" t="n">
         <v>0</v>
       </c>
+      <c r="G18" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -951,6 +1019,9 @@
       <c r="F19" t="n">
         <v>1</v>
       </c>
+      <c r="G19" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -979,6 +1050,9 @@
       <c r="F20" t="n">
         <v>1</v>
       </c>
+      <c r="G20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1007,6 +1081,9 @@
       <c r="F21" t="n">
         <v>1</v>
       </c>
+      <c r="G21" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1035,6 +1112,9 @@
       <c r="F22" t="n">
         <v>0</v>
       </c>
+      <c r="G22" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1063,6 +1143,9 @@
       <c r="F23" t="n">
         <v>0</v>
       </c>
+      <c r="G23" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1091,6 +1174,9 @@
       <c r="F24" t="n">
         <v>0</v>
       </c>
+      <c r="G24" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1119,6 +1205,9 @@
       <c r="F25" t="n">
         <v>0</v>
       </c>
+      <c r="G25" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1147,6 +1236,9 @@
       <c r="F26" t="n">
         <v>0</v>
       </c>
+      <c r="G26" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1175,6 +1267,9 @@
       <c r="F27" t="n">
         <v>0</v>
       </c>
+      <c r="G27" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1203,6 +1298,9 @@
       <c r="F28" t="n">
         <v>1</v>
       </c>
+      <c r="G28" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1231,6 +1329,9 @@
       <c r="F29" t="n">
         <v>1</v>
       </c>
+      <c r="G29" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1259,6 +1360,9 @@
       <c r="F30" t="n">
         <v>0</v>
       </c>
+      <c r="G30" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1287,6 +1391,9 @@
       <c r="F31" t="n">
         <v>1</v>
       </c>
+      <c r="G31" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1315,6 +1422,9 @@
       <c r="F32" t="n">
         <v>0</v>
       </c>
+      <c r="G32" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1343,6 +1453,9 @@
       <c r="F33" t="n">
         <v>0</v>
       </c>
+      <c r="G33" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1371,6 +1484,9 @@
       <c r="F34" t="n">
         <v>0</v>
       </c>
+      <c r="G34" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1399,6 +1515,9 @@
       <c r="F35" t="n">
         <v>0</v>
       </c>
+      <c r="G35" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1427,6 +1546,9 @@
       <c r="F36" t="n">
         <v>0</v>
       </c>
+      <c r="G36" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1455,6 +1577,9 @@
       <c r="F37" t="n">
         <v>1</v>
       </c>
+      <c r="G37" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1483,6 +1608,9 @@
       <c r="F38" t="n">
         <v>0</v>
       </c>
+      <c r="G38" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1511,6 +1639,9 @@
       <c r="F39" t="n">
         <v>0</v>
       </c>
+      <c r="G39" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1539,6 +1670,9 @@
       <c r="F40" t="n">
         <v>0</v>
       </c>
+      <c r="G40" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1567,6 +1701,9 @@
       <c r="F41" t="n">
         <v>0</v>
       </c>
+      <c r="G41" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1595,6 +1732,9 @@
       <c r="F42" t="n">
         <v>0</v>
       </c>
+      <c r="G42" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1623,6 +1763,9 @@
       <c r="F43" t="n">
         <v>0</v>
       </c>
+      <c r="G43" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1651,6 +1794,9 @@
       <c r="F44" t="n">
         <v>1</v>
       </c>
+      <c r="G44" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1677,6 +1823,9 @@
         </is>
       </c>
       <c r="F45" t="n">
+        <v>0</v>
+      </c>
+      <c r="G45" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>